<commit_message>
update processed data 4
</commit_message>
<xml_diff>
--- a/data/metadata/ANON-ptcp-log.xlsx
+++ b/data/metadata/ANON-ptcp-log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/babylab/General Lab Resources/Studies/LexVar/4_writing/gh/LexVar/data/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F73D119C-BE53-0A49-B41C-7B3A4C6C24CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3DCC26B-8266-5944-AFEA-C85C54C3D197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="280" yWindow="500" windowWidth="18420" windowHeight="13260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39060" yWindow="-100" windowWidth="21940" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v1" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="558" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="123">
   <si>
     <t>ptcp_id</t>
   </si>
@@ -148,9 +148,6 @@
     <t>ethnicity</t>
   </si>
   <si>
-    <t>eng</t>
-  </si>
-  <si>
     <t>white</t>
   </si>
   <si>
@@ -376,37 +373,43 @@
     <t>p190</t>
   </si>
   <si>
+    <t>p188</t>
+  </si>
+  <si>
+    <t>p191</t>
+  </si>
+  <si>
+    <t>exclusion_reason</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>age_d</t>
+  </si>
+  <si>
+    <t>failed calibration</t>
+  </si>
+  <si>
+    <t>insufficient trials</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>family interruption</t>
+  </si>
+  <si>
+    <t>refused to sit on caregiver's lap</t>
+  </si>
+  <si>
+    <t>double recruited</t>
+  </si>
+  <si>
+    <t>refused to wear sticker</t>
+  </si>
+  <si>
     <t>did not meet language requirement</t>
-  </si>
-  <si>
-    <t>&lt;80</t>
-  </si>
-  <si>
-    <t>p188</t>
-  </si>
-  <si>
-    <t>p191</t>
-  </si>
-  <si>
-    <t>exclusion_reason</t>
-  </si>
-  <si>
-    <t>age</t>
-  </si>
-  <si>
-    <t>age_d</t>
-  </si>
-  <si>
-    <t>failed calibration</t>
-  </si>
-  <si>
-    <t>insufficient trials</t>
-  </si>
-  <si>
-    <t>n/a</t>
-  </si>
-  <si>
-    <t>family interruption</t>
   </si>
 </sst>
 </file>
@@ -765,16 +768,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K92"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" style="3" customWidth="1"/>
-    <col min="5" max="9" width="10.83203125" customWidth="1"/>
+    <col min="5" max="8" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -785,31 +788,28 @@
         <v>1</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E1" t="s">
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="I1" t="s">
+        <v>29</v>
+      </c>
       <c r="J1" t="s">
-        <v>29</v>
-      </c>
-      <c r="K1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -829,22 +829,19 @@
         <v>13</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H2" s="1">
-        <v>100</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" t="s">
-        <v>6</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I2" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -864,22 +861,19 @@
         <v>14</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H3" s="1">
-        <v>100</v>
+        <v>35</v>
+      </c>
+      <c r="H3" t="s">
+        <v>11</v>
       </c>
       <c r="I3" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J3" t="s">
-        <v>6</v>
-      </c>
-      <c r="K3" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -899,22 +893,19 @@
         <v>7</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H4" s="1">
-        <v>100</v>
+        <v>39</v>
+      </c>
+      <c r="H4" t="s">
+        <v>8</v>
       </c>
       <c r="I4" t="s">
         <v>8</v>
       </c>
       <c r="J4" t="s">
-        <v>8</v>
-      </c>
-      <c r="K4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -934,22 +925,19 @@
         <v>14</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="1">
-        <v>100</v>
+        <v>35</v>
+      </c>
+      <c r="H5" t="s">
+        <v>8</v>
       </c>
       <c r="I5" t="s">
         <v>8</v>
       </c>
       <c r="J5" t="s">
-        <v>8</v>
-      </c>
-      <c r="K5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -969,22 +957,19 @@
         <v>9</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="1">
-        <v>100</v>
+        <v>39</v>
+      </c>
+      <c r="H6" t="s">
+        <v>11</v>
       </c>
       <c r="I6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J6" t="s">
-        <v>6</v>
-      </c>
-      <c r="K6" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -1004,22 +989,19 @@
         <v>24</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="H7" s="1">
-        <v>90</v>
+        <v>41</v>
+      </c>
+      <c r="H7" t="s">
+        <v>11</v>
       </c>
       <c r="I7" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J7" t="s">
-        <v>8</v>
-      </c>
-      <c r="K7" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1039,22 +1021,19 @@
         <v>12</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H8" s="1">
-        <v>80</v>
+        <v>40</v>
+      </c>
+      <c r="H8" t="s">
+        <v>8</v>
       </c>
       <c r="I8" t="s">
         <v>8</v>
       </c>
       <c r="J8" t="s">
-        <v>8</v>
-      </c>
-      <c r="K8" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1074,22 +1053,19 @@
         <v>7</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H9" s="1">
-        <v>100</v>
+        <v>35</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
       </c>
       <c r="I9" t="s">
         <v>6</v>
       </c>
       <c r="J9" t="s">
-        <v>6</v>
-      </c>
-      <c r="K9" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1109,22 +1085,19 @@
         <v>11</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H10" s="1">
-        <v>99</v>
+        <v>39</v>
+      </c>
+      <c r="H10" t="s">
+        <v>6</v>
       </c>
       <c r="I10" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J10" t="s">
-        <v>8</v>
-      </c>
-      <c r="K10" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1144,22 +1117,19 @@
         <v>7</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H11" s="1">
-        <v>100</v>
+        <v>39</v>
+      </c>
+      <c r="H11" t="s">
+        <v>8</v>
       </c>
       <c r="I11" t="s">
         <v>8</v>
       </c>
       <c r="J11" t="s">
-        <v>8</v>
-      </c>
-      <c r="K11" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1179,22 +1149,19 @@
         <v>21</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H12" s="1">
-        <v>100</v>
+        <v>35</v>
+      </c>
+      <c r="H12" t="s">
+        <v>6</v>
       </c>
       <c r="I12" t="s">
         <v>6</v>
       </c>
       <c r="J12" t="s">
-        <v>6</v>
-      </c>
-      <c r="K12" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1214,22 +1181,19 @@
         <v>17</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H13" s="1">
-        <v>95</v>
+        <v>35</v>
+      </c>
+      <c r="H13" t="s">
+        <v>11</v>
       </c>
       <c r="I13" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J13" t="s">
-        <v>8</v>
-      </c>
-      <c r="K13" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1249,22 +1213,19 @@
         <v>7</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H14" s="1">
-        <v>100</v>
+        <v>37</v>
+      </c>
+      <c r="H14" t="s">
+        <v>11</v>
       </c>
       <c r="I14" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J14" t="s">
-        <v>6</v>
-      </c>
-      <c r="K14" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1284,22 +1245,19 @@
         <v>4</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H15" s="1">
-        <v>100</v>
+        <v>39</v>
+      </c>
+      <c r="H15" t="s">
+        <v>11</v>
       </c>
       <c r="I15" t="s">
         <v>6</v>
       </c>
       <c r="J15" t="s">
-        <v>6</v>
-      </c>
-      <c r="K15" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1319,22 +1277,19 @@
         <v>24</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H16" s="1">
-        <v>95</v>
+        <v>40</v>
+      </c>
+      <c r="H16" t="s">
+        <v>11</v>
       </c>
       <c r="I16" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="J16" t="s">
-        <v>6</v>
-      </c>
-      <c r="K16" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -1354,22 +1309,19 @@
         <v>30</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H17" s="1">
-        <v>85</v>
+        <v>35</v>
+      </c>
+      <c r="H17" t="s">
+        <v>8</v>
       </c>
       <c r="I17" t="s">
         <v>8</v>
       </c>
       <c r="J17" t="s">
-        <v>6</v>
-      </c>
-      <c r="K17" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -1389,22 +1341,19 @@
         <v>18</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H18" s="1">
-        <v>100</v>
+        <v>35</v>
+      </c>
+      <c r="H18" t="s">
+        <v>11</v>
       </c>
       <c r="I18" t="s">
         <v>8</v>
       </c>
       <c r="J18" t="s">
-        <v>6</v>
-      </c>
-      <c r="K18" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1424,22 +1373,19 @@
         <v>7</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H19" s="1">
-        <v>100</v>
+        <v>37</v>
+      </c>
+      <c r="H19" t="s">
+        <v>8</v>
       </c>
       <c r="I19" t="s">
         <v>8</v>
       </c>
       <c r="J19" t="s">
-        <v>8</v>
-      </c>
-      <c r="K19" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -1459,22 +1405,19 @@
         <v>5</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H20" s="1">
-        <v>100</v>
+        <v>35</v>
+      </c>
+      <c r="H20" t="s">
+        <v>8</v>
       </c>
       <c r="I20" t="s">
         <v>8</v>
       </c>
       <c r="J20" t="s">
-        <v>8</v>
-      </c>
-      <c r="K20" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1494,22 +1437,19 @@
         <v>16</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H21" s="1">
-        <v>100</v>
+        <v>36</v>
+      </c>
+      <c r="H21" t="s">
+        <v>6</v>
       </c>
       <c r="I21" t="s">
         <v>6</v>
       </c>
       <c r="J21" t="s">
-        <v>6</v>
-      </c>
-      <c r="K21" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -1529,22 +1469,19 @@
         <v>12</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H22" s="1">
-        <v>100</v>
+        <v>35</v>
+      </c>
+      <c r="H22" t="s">
+        <v>8</v>
       </c>
       <c r="I22" t="s">
         <v>8</v>
       </c>
       <c r="J22" t="s">
-        <v>8</v>
-      </c>
-      <c r="K22" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -1564,24 +1501,21 @@
         <v>12</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H23" s="1">
-        <v>100</v>
+        <v>38</v>
+      </c>
+      <c r="H23" t="s">
+        <v>6</v>
       </c>
       <c r="I23" t="s">
         <v>6</v>
       </c>
       <c r="J23" t="s">
-        <v>6</v>
-      </c>
-      <c r="K23" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B24">
         <v>5</v>
@@ -1599,24 +1533,21 @@
         <v>27</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H24" s="1">
-        <v>100</v>
-      </c>
-      <c r="I24" t="s">
-        <v>11</v>
+        <v>35</v>
+      </c>
+      <c r="H24" t="s">
+        <v>6</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K24" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B25">
         <v>6</v>
@@ -1634,24 +1565,21 @@
         <v>19</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H25" s="1">
-        <v>100</v>
-      </c>
-      <c r="I25" t="s">
-        <v>11</v>
+        <v>35</v>
+      </c>
+      <c r="H25" t="s">
+        <v>6</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K25" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B26">
         <v>7</v>
@@ -1669,24 +1597,21 @@
         <v>24</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H26" s="1">
-        <v>100</v>
+        <v>35</v>
+      </c>
+      <c r="H26" t="s">
+        <v>6</v>
       </c>
       <c r="I26" t="s">
         <v>6</v>
       </c>
       <c r="J26" t="s">
-        <v>6</v>
-      </c>
-      <c r="K26" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B27">
         <v>8</v>
@@ -1704,24 +1629,21 @@
         <v>17</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H27" s="1">
-        <v>99</v>
-      </c>
-      <c r="I27" t="s">
+        <v>35</v>
+      </c>
+      <c r="H27" t="s">
+        <v>8</v>
+      </c>
+      <c r="I27" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B28">
         <v>9</v>
@@ -1739,24 +1661,21 @@
         <v>10</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H28" s="1">
-        <v>99.9</v>
-      </c>
-      <c r="I28" t="s">
+        <v>35</v>
+      </c>
+      <c r="H28" t="s">
+        <v>8</v>
+      </c>
+      <c r="I28" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K28" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B29">
         <v>10</v>
@@ -1774,24 +1693,21 @@
         <v>19</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H29" s="1">
-        <v>85</v>
-      </c>
-      <c r="I29" t="s">
+        <v>50</v>
+      </c>
+      <c r="H29" t="s">
+        <v>11</v>
+      </c>
+      <c r="I29" s="1" t="s">
         <v>6</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B30">
         <v>11</v>
@@ -1809,24 +1725,21 @@
         <v>19</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H30" s="1">
-        <v>100</v>
-      </c>
-      <c r="I30" t="s">
+        <v>35</v>
+      </c>
+      <c r="H30" t="s">
+        <v>8</v>
+      </c>
+      <c r="I30" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K30" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B31">
         <v>12</v>
@@ -1844,24 +1757,21 @@
         <v>8</v>
       </c>
       <c r="G31" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H31" t="s">
+        <v>11</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
         <v>51</v>
-      </c>
-      <c r="H31" s="1">
-        <v>100</v>
-      </c>
-      <c r="I31" t="s">
-        <v>8</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>52</v>
       </c>
       <c r="B32">
         <v>13</v>
@@ -1879,24 +1789,21 @@
         <v>18</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H32" s="1">
-        <v>100</v>
-      </c>
-      <c r="I32" t="s">
+        <v>35</v>
+      </c>
+      <c r="H32" t="s">
         <v>11</v>
       </c>
+      <c r="I32" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="J32" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K32" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B33">
         <v>14</v>
@@ -1914,24 +1821,21 @@
         <v>3</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H33" s="1">
-        <v>95</v>
-      </c>
-      <c r="I33" t="s">
-        <v>8</v>
+        <v>40</v>
+      </c>
+      <c r="H33" t="s">
+        <v>6</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K33" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B34">
         <v>15</v>
@@ -1949,24 +1853,21 @@
         <v>4</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H34" s="1">
-        <v>100</v>
-      </c>
-      <c r="I34" t="s">
+        <v>40</v>
+      </c>
+      <c r="H34" t="s">
+        <v>8</v>
+      </c>
+      <c r="I34" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K34" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B35">
         <v>16</v>
@@ -1984,24 +1885,21 @@
         <v>29</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H35" s="1">
-        <v>95</v>
-      </c>
-      <c r="I35" t="s">
+        <v>39</v>
+      </c>
+      <c r="H35" t="s">
+        <v>11</v>
+      </c>
+      <c r="I35" s="1" t="s">
         <v>6</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K35" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B36">
         <v>17</v>
@@ -2019,24 +1917,21 @@
         <v>2</v>
       </c>
       <c r="G36" t="s">
-        <v>40</v>
-      </c>
-      <c r="H36" s="1">
-        <v>100</v>
-      </c>
-      <c r="I36" t="s">
+        <v>39</v>
+      </c>
+      <c r="H36" t="s">
         <v>11</v>
       </c>
+      <c r="I36" s="1" t="s">
+        <v>6</v>
+      </c>
       <c r="J36" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K36" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B37">
         <v>18</v>
@@ -2054,24 +1949,21 @@
         <v>6</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H37" s="1">
-        <v>100</v>
-      </c>
-      <c r="I37" t="s">
-        <v>19</v>
+        <v>35</v>
+      </c>
+      <c r="H37" t="s">
+        <v>6</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K37" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B38">
         <v>1</v>
@@ -2089,24 +1981,21 @@
         <v>19</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H38" s="1">
-        <v>100</v>
-      </c>
-      <c r="I38" t="s">
+        <v>35</v>
+      </c>
+      <c r="H38" t="s">
+        <v>8</v>
+      </c>
+      <c r="I38" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K38" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B39">
         <v>2</v>
@@ -2124,24 +2013,21 @@
         <v>9</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H39" s="1">
-        <v>90</v>
-      </c>
-      <c r="I39" t="s">
+        <v>50</v>
+      </c>
+      <c r="H39" t="s">
+        <v>8</v>
+      </c>
+      <c r="I39" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K39" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B40">
         <v>3</v>
@@ -2159,24 +2045,21 @@
         <v>16</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H40" s="1">
-        <v>100</v>
-      </c>
-      <c r="I40" t="s">
+        <v>35</v>
+      </c>
+      <c r="H40" t="s">
+        <v>8</v>
+      </c>
+      <c r="I40" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K40" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B41">
         <v>4</v>
@@ -2194,24 +2077,21 @@
         <v>26</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H41" s="1">
-        <v>99</v>
-      </c>
-      <c r="I41" t="s">
+        <v>40</v>
+      </c>
+      <c r="H41" t="s">
+        <v>8</v>
+      </c>
+      <c r="I41" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K41" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B42">
         <v>5</v>
@@ -2229,24 +2109,21 @@
         <v>17</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H42" s="1">
-        <v>100</v>
-      </c>
-      <c r="I42" t="s">
+        <v>35</v>
+      </c>
+      <c r="H42" t="s">
+        <v>8</v>
+      </c>
+      <c r="I42" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K42" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B43">
         <v>6</v>
@@ -2264,24 +2141,21 @@
         <v>3</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H43" s="1">
-        <v>100</v>
-      </c>
-      <c r="I43" t="s">
+        <v>35</v>
+      </c>
+      <c r="H43" t="s">
+        <v>8</v>
+      </c>
+      <c r="I43" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K43" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B44">
         <v>7</v>
@@ -2299,24 +2173,21 @@
         <v>4</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H44" s="1">
-        <v>100</v>
-      </c>
-      <c r="I44" t="s">
-        <v>8</v>
+        <v>39</v>
+      </c>
+      <c r="H44" t="s">
+        <v>6</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K44" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B45">
         <v>8</v>
@@ -2334,24 +2205,21 @@
         <v>30</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H45" s="1">
-        <v>100</v>
-      </c>
-      <c r="I45" t="s">
+        <v>35</v>
+      </c>
+      <c r="H45" t="s">
+        <v>8</v>
+      </c>
+      <c r="I45" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K45" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B46">
         <v>9</v>
@@ -2369,24 +2237,21 @@
         <v>20</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H46" s="1">
-        <v>95</v>
-      </c>
-      <c r="I46" t="s">
-        <v>11</v>
+        <v>35</v>
+      </c>
+      <c r="H46" t="s">
+        <v>6</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K46" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B47">
         <v>10</v>
@@ -2404,24 +2269,21 @@
         <v>12</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H47" s="1">
-        <v>85</v>
-      </c>
-      <c r="I47" t="s">
+        <v>39</v>
+      </c>
+      <c r="H47" t="s">
+        <v>8</v>
+      </c>
+      <c r="I47" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K47" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B48">
         <v>11</v>
@@ -2439,24 +2301,21 @@
         <v>13</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H48" s="1">
-        <v>95</v>
-      </c>
-      <c r="I48" t="s">
+        <v>50</v>
+      </c>
+      <c r="H48" t="s">
+        <v>6</v>
+      </c>
+      <c r="I48" s="1" t="s">
         <v>6</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K48" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B49">
         <v>12</v>
@@ -2474,24 +2333,21 @@
         <v>1</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H49" s="1">
-        <v>100</v>
-      </c>
-      <c r="I49" t="s">
-        <v>11</v>
+        <v>35</v>
+      </c>
+      <c r="H49" t="s">
+        <v>6</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K49" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B50">
         <v>13</v>
@@ -2509,24 +2365,21 @@
         <v>16</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H50" s="1">
-        <v>100</v>
-      </c>
-      <c r="I50" t="s">
-        <v>19</v>
+        <v>39</v>
+      </c>
+      <c r="H50" t="s">
+        <v>11</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>8</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K50" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B51">
         <v>14</v>
@@ -2544,24 +2397,21 @@
         <v>11</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H51" s="1">
-        <v>100</v>
-      </c>
-      <c r="I51" t="s">
+        <v>35</v>
+      </c>
+      <c r="H51" t="s">
         <v>19</v>
       </c>
+      <c r="I51" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="J51" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K51" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B52">
         <v>15</v>
@@ -2579,24 +2429,21 @@
         <v>7</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H52" s="1">
-        <v>100</v>
-      </c>
-      <c r="I52" t="s">
+        <v>35</v>
+      </c>
+      <c r="H52" t="s">
+        <v>8</v>
+      </c>
+      <c r="I52" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K52" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B53">
         <v>16</v>
@@ -2614,24 +2461,21 @@
         <v>2</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H53" s="1">
-        <v>100</v>
-      </c>
-      <c r="I53" t="s">
-        <v>11</v>
+        <v>39</v>
+      </c>
+      <c r="H53" t="s">
+        <v>6</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J53" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K53" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B54">
         <v>17</v>
@@ -2649,24 +2493,21 @@
         <v>8</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H54" s="1">
-        <v>98</v>
-      </c>
-      <c r="I54" t="s">
+        <v>50</v>
+      </c>
+      <c r="H54" t="s">
+        <v>8</v>
+      </c>
+      <c r="I54" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K54" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B55">
         <v>18</v>
@@ -2684,24 +2525,21 @@
         <v>2</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H55" s="1">
-        <v>100</v>
-      </c>
-      <c r="I55" t="s">
+        <v>39</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J55" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K55" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B56">
         <v>1</v>
@@ -2719,24 +2557,21 @@
         <v>12</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H56" s="1">
-        <v>100</v>
-      </c>
-      <c r="I56" t="s">
+        <v>50</v>
+      </c>
+      <c r="H56" t="s">
+        <v>8</v>
+      </c>
+      <c r="I56" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K56" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B57">
         <v>2</v>
@@ -2754,24 +2589,21 @@
         <v>12</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H57" s="1">
-        <v>100</v>
-      </c>
-      <c r="I57" t="s">
+        <v>39</v>
+      </c>
+      <c r="H57" t="s">
         <v>19</v>
       </c>
+      <c r="I57" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="J57" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K57" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B58">
         <v>3</v>
@@ -2789,24 +2621,21 @@
         <v>2</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H58" s="1">
-        <v>100</v>
-      </c>
-      <c r="I58" t="s">
+        <v>39</v>
+      </c>
+      <c r="H58" t="s">
+        <v>8</v>
+      </c>
+      <c r="I58" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K58" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B59">
         <v>4</v>
@@ -2824,24 +2653,21 @@
         <v>18</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H59" s="1">
-        <v>100</v>
-      </c>
-      <c r="I59" t="s">
-        <v>19</v>
+        <v>35</v>
+      </c>
+      <c r="H59" t="s">
+        <v>6</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J59" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K59" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B60">
         <v>5</v>
@@ -2859,24 +2685,21 @@
         <v>30</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H60" s="1">
-        <v>100</v>
-      </c>
-      <c r="I60" t="s">
+        <v>35</v>
+      </c>
+      <c r="H60" t="s">
+        <v>8</v>
+      </c>
+      <c r="I60" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K60" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B61">
         <v>6</v>
@@ -2894,24 +2717,21 @@
         <v>3</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H61" s="1">
-        <v>90</v>
-      </c>
-      <c r="I61" t="s">
+        <v>50</v>
+      </c>
+      <c r="H61" t="s">
         <v>19</v>
       </c>
+      <c r="I61" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="J61" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K61" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B62">
         <v>7</v>
@@ -2929,24 +2749,21 @@
         <v>0</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H62" s="1">
-        <v>100</v>
-      </c>
-      <c r="I62" t="s">
-        <v>19</v>
+        <v>35</v>
+      </c>
+      <c r="H62" t="s">
+        <v>6</v>
+      </c>
+      <c r="I62" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J62" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K62" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B63">
         <v>8</v>
@@ -2964,24 +2781,21 @@
         <v>7</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H63" s="1">
-        <v>100</v>
-      </c>
-      <c r="I63" t="s">
+        <v>35</v>
+      </c>
+      <c r="H63" t="s">
+        <v>8</v>
+      </c>
+      <c r="I63" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K63" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B64">
         <v>9</v>
@@ -2999,24 +2813,21 @@
         <v>18</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H64" s="1">
-        <v>100</v>
-      </c>
-      <c r="I64" t="s">
+        <v>39</v>
+      </c>
+      <c r="H64" t="s">
+        <v>8</v>
+      </c>
+      <c r="I64" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K64" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B65">
         <v>10</v>
@@ -3034,24 +2845,21 @@
         <v>15</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H65" s="1">
-        <v>100</v>
-      </c>
-      <c r="I65" t="s">
+        <v>50</v>
+      </c>
+      <c r="H65" t="s">
+        <v>6</v>
+      </c>
+      <c r="I65" s="1" t="s">
         <v>6</v>
       </c>
       <c r="J65" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K65" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B66">
         <v>11</v>
@@ -3069,24 +2877,21 @@
         <v>24</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H66" s="1">
-        <v>100</v>
-      </c>
-      <c r="I66" t="s">
+        <v>35</v>
+      </c>
+      <c r="H66" t="s">
+        <v>8</v>
+      </c>
+      <c r="I66" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K66" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B67">
         <v>12</v>
@@ -3104,24 +2909,21 @@
         <v>20</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H67" s="1">
-        <v>100</v>
-      </c>
-      <c r="I67" t="s">
+        <v>36</v>
+      </c>
+      <c r="H67" t="s">
         <v>11</v>
       </c>
+      <c r="I67" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="J67" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B68">
         <v>13</v>
@@ -3139,24 +2941,21 @@
         <v>9</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H68" s="1">
-        <v>90</v>
-      </c>
-      <c r="I68" t="s">
-        <v>11</v>
+        <v>40</v>
+      </c>
+      <c r="H68" t="s">
+        <v>6</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J68" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K68" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B69">
         <v>14</v>
@@ -3174,24 +2973,21 @@
         <v>4</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H69" s="1">
-        <v>100</v>
-      </c>
-      <c r="I69" t="s">
-        <v>11</v>
+        <v>35</v>
+      </c>
+      <c r="H69" t="s">
+        <v>6</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J69" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B70">
         <v>15</v>
@@ -3209,24 +3005,21 @@
         <v>21</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H70" s="1">
-        <v>100</v>
-      </c>
-      <c r="I70" t="s">
+        <v>50</v>
+      </c>
+      <c r="H70" t="s">
+        <v>8</v>
+      </c>
+      <c r="I70" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J70" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B71">
         <v>16</v>
@@ -3244,24 +3037,21 @@
         <v>1</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H71" s="1">
-        <v>80</v>
-      </c>
-      <c r="I71" t="s">
+        <v>50</v>
+      </c>
+      <c r="H71" t="s">
+        <v>8</v>
+      </c>
+      <c r="I71" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J71" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K71" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B72">
         <v>17</v>
@@ -3279,24 +3069,21 @@
         <v>21</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H72" s="1">
-        <v>100</v>
-      </c>
-      <c r="I72" t="s">
+        <v>40</v>
+      </c>
+      <c r="H72" t="s">
+        <v>8</v>
+      </c>
+      <c r="I72" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J72" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B73">
         <v>18</v>
@@ -3314,24 +3101,21 @@
         <v>12</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H73" s="1">
-        <v>100</v>
-      </c>
-      <c r="I73" t="s">
+        <v>35</v>
+      </c>
+      <c r="H73" t="s">
+        <v>8</v>
+      </c>
+      <c r="I73" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B74">
         <v>1</v>
@@ -3349,24 +3133,21 @@
         <v>24</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H74" s="1">
-        <v>80</v>
-      </c>
-      <c r="I74" t="s">
+        <v>50</v>
+      </c>
+      <c r="H74" t="s">
         <v>19</v>
       </c>
+      <c r="I74" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="J74" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K74" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B75">
         <v>2</v>
@@ -3384,24 +3165,21 @@
         <v>16</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H75" s="1">
-        <v>100</v>
-      </c>
-      <c r="I75" t="s">
+        <v>35</v>
+      </c>
+      <c r="H75" t="s">
+        <v>11</v>
+      </c>
+      <c r="I75" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J75" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K75" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B76">
         <v>3</v>
@@ -3419,24 +3197,21 @@
         <v>26</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H76" s="1">
-        <v>100</v>
-      </c>
-      <c r="I76" t="s">
+        <v>39</v>
+      </c>
+      <c r="H76" t="s">
         <v>19</v>
       </c>
+      <c r="I76" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="J76" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K76" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B77">
         <v>4</v>
@@ -3454,24 +3229,21 @@
         <v>26</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H77" s="1">
-        <v>80</v>
-      </c>
-      <c r="I77" t="s">
+        <v>50</v>
+      </c>
+      <c r="H77" t="s">
+        <v>8</v>
+      </c>
+      <c r="I77" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J77" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K77" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B78">
         <v>5</v>
@@ -3489,24 +3261,21 @@
         <v>30</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H78" s="1">
-        <v>100</v>
-      </c>
-      <c r="I78" t="s">
+        <v>50</v>
+      </c>
+      <c r="H78" t="s">
+        <v>8</v>
+      </c>
+      <c r="I78" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J78" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K78" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B79">
         <v>6</v>
@@ -3524,24 +3293,21 @@
         <v>2</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H79" s="1">
-        <v>100</v>
-      </c>
-      <c r="I79" t="s">
+        <v>35</v>
+      </c>
+      <c r="H79" t="s">
+        <v>8</v>
+      </c>
+      <c r="I79" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J79" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K79" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B80">
         <v>7</v>
@@ -3559,24 +3325,21 @@
         <v>0</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H80" s="1">
+        <v>35</v>
+      </c>
+      <c r="H80" t="s">
+        <v>8</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J80" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
         <v>100</v>
-      </c>
-      <c r="I80" t="s">
-        <v>8</v>
-      </c>
-      <c r="J80" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K80" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A81" t="s">
-        <v>101</v>
       </c>
       <c r="B81">
         <v>8</v>
@@ -3594,24 +3357,21 @@
         <v>9</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H81" s="1">
-        <v>100</v>
-      </c>
-      <c r="I81" t="s">
+        <v>35</v>
+      </c>
+      <c r="H81" t="s">
+        <v>8</v>
+      </c>
+      <c r="I81" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J81" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K81" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B82">
         <v>9</v>
@@ -3629,24 +3389,21 @@
         <v>28</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H82" s="1">
-        <v>95</v>
-      </c>
-      <c r="I82" t="s">
+        <v>40</v>
+      </c>
+      <c r="H82" t="s">
+        <v>8</v>
+      </c>
+      <c r="I82" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K82" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B83">
         <v>10</v>
@@ -3664,24 +3421,21 @@
         <v>10</v>
       </c>
       <c r="G83" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H83" s="1">
-        <v>90</v>
-      </c>
-      <c r="I83" t="s">
+        <v>39</v>
+      </c>
+      <c r="H83" t="s">
         <v>19</v>
       </c>
+      <c r="I83" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="J83" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K83" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B84">
         <v>11</v>
@@ -3699,24 +3453,21 @@
         <v>25</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H84" s="1">
-        <v>99</v>
-      </c>
-      <c r="I84" t="s">
-        <v>19</v>
+        <v>39</v>
+      </c>
+      <c r="H84" t="s">
+        <v>6</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>6</v>
       </c>
       <c r="J84" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K84" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B85">
         <v>12</v>
@@ -3734,24 +3485,21 @@
         <v>10</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H85" s="1">
-        <v>100</v>
-      </c>
-      <c r="I85" t="s">
+        <v>35</v>
+      </c>
+      <c r="H85" t="s">
+        <v>8</v>
+      </c>
+      <c r="I85" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J85" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K85" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B86">
         <v>13</v>
@@ -3769,24 +3517,21 @@
         <v>3</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H86" s="1">
-        <v>100</v>
-      </c>
-      <c r="I86" t="s">
+        <v>35</v>
+      </c>
+      <c r="H86" t="s">
+        <v>8</v>
+      </c>
+      <c r="I86" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J86" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K86" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B87">
         <v>14</v>
@@ -3804,24 +3549,21 @@
         <v>12</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H87" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="I87" t="s">
+        <v>40</v>
+      </c>
+      <c r="H87" t="s">
+        <v>6</v>
+      </c>
+      <c r="I87" s="1" t="s">
         <v>6</v>
       </c>
       <c r="J87" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K87" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B88">
         <v>15</v>
@@ -3839,24 +3581,21 @@
         <v>24</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H88" s="1">
-        <v>80</v>
-      </c>
-      <c r="I88" t="s">
+        <v>35</v>
+      </c>
+      <c r="H88" t="s">
+        <v>6</v>
+      </c>
+      <c r="I88" s="1" t="s">
         <v>6</v>
       </c>
       <c r="J88" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K88" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B89">
         <v>16</v>
@@ -3874,24 +3613,21 @@
         <v>20</v>
       </c>
       <c r="G89" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H89" s="1">
-        <v>90</v>
-      </c>
-      <c r="I89" t="s">
-        <v>19</v>
+        <v>50</v>
+      </c>
+      <c r="H89" t="s">
+        <v>11</v>
+      </c>
+      <c r="I89" s="1" t="s">
+        <v>8</v>
       </c>
       <c r="J89" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K89" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B90">
         <v>17</v>
@@ -3909,24 +3645,21 @@
         <v>6</v>
       </c>
       <c r="G90" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H90" s="1">
-        <v>100</v>
-      </c>
-      <c r="I90" t="s">
+        <v>35</v>
+      </c>
+      <c r="H90" t="s">
         <v>19</v>
       </c>
+      <c r="I90" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="J90" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K90" s="1" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B91">
         <v>18</v>
@@ -3944,24 +3677,21 @@
         <v>23</v>
       </c>
       <c r="G91" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H91" s="1">
-        <v>100</v>
-      </c>
-      <c r="I91" t="s">
+        <v>35</v>
+      </c>
+      <c r="H91" t="s">
+        <v>8</v>
+      </c>
+      <c r="I91" s="1" t="s">
         <v>8</v>
       </c>
       <c r="J91" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K91" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B92">
         <v>1</v>
@@ -3979,19 +3709,16 @@
         <v>22</v>
       </c>
       <c r="G92" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H92" s="1">
-        <v>100</v>
-      </c>
-      <c r="I92" t="s">
+        <v>36</v>
+      </c>
+      <c r="H92" t="s">
         <v>19</v>
       </c>
+      <c r="I92" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="J92" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K92" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add education + small edits
</commit_message>
<xml_diff>
--- a/data/metadata/ANON-ptcp-log.xlsx
+++ b/data/metadata/ANON-ptcp-log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/babylab/General Lab Resources/Studies/LexVar/4_writing/gh/LexVar/data/metadata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kcasey/Desktop/LexVar/data/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3DCC26B-8266-5944-AFEA-C85C54C3D197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22AD0C8C-4B8E-5A4D-9626-4A78342B098A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39060" yWindow="-100" windowWidth="21940" windowHeight="15820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="-2080" windowWidth="38400" windowHeight="21600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="v1" sheetId="2" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="129">
   <si>
     <t>ptcp_id</t>
   </si>
@@ -410,6 +410,24 @@
   </si>
   <si>
     <t>did not meet language requirement</t>
+  </si>
+  <si>
+    <t>maternal_education</t>
+  </si>
+  <si>
+    <t>master's</t>
+  </si>
+  <si>
+    <t>terminal degree</t>
+  </si>
+  <si>
+    <t>bachelor's</t>
+  </si>
+  <si>
+    <t>some college</t>
+  </si>
+  <si>
+    <t>high school</t>
   </si>
 </sst>
 </file>
@@ -768,16 +786,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J92"/>
+  <dimension ref="A1:K92"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="10.83203125" style="3" customWidth="1"/>
-    <col min="5" max="8" width="10.83203125" customWidth="1"/>
+    <col min="5" max="7" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -800,16 +819,19 @@
         <v>34</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>29</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -832,16 +854,19 @@
         <v>35</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I2" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K2" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -863,17 +888,20 @@
       <c r="G3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I3" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s">
-        <v>6</v>
-      </c>
       <c r="J3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K3" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -895,17 +923,20 @@
       <c r="G4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H4" t="s">
-        <v>8</v>
+      <c r="H4" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="I4" t="s">
         <v>8</v>
       </c>
       <c r="J4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -927,17 +958,20 @@
       <c r="G5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H5" t="s">
-        <v>8</v>
+      <c r="H5" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="I5" t="s">
         <v>8</v>
       </c>
       <c r="J5" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K5" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -959,17 +993,20 @@
       <c r="G6" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I6" t="s">
         <v>11</v>
       </c>
-      <c r="I6" t="s">
-        <v>8</v>
-      </c>
       <c r="J6" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -991,17 +1028,20 @@
       <c r="G7" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I7" t="s">
         <v>11</v>
       </c>
-      <c r="I7" t="s">
-        <v>8</v>
-      </c>
       <c r="J7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1023,17 +1063,20 @@
       <c r="G8" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H8" t="s">
-        <v>8</v>
+      <c r="H8" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="I8" t="s">
         <v>8</v>
       </c>
       <c r="J8" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1055,17 +1098,20 @@
       <c r="G9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" t="s">
         <v>11</v>
       </c>
-      <c r="I9" t="s">
-        <v>6</v>
-      </c>
       <c r="J9" t="s">
+        <v>6</v>
+      </c>
+      <c r="K9" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1087,17 +1133,20 @@
       <c r="G10" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H10" t="s">
-        <v>6</v>
+      <c r="H10" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="I10" t="s">
         <v>6</v>
       </c>
       <c r="J10" t="s">
+        <v>6</v>
+      </c>
+      <c r="K10" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -1119,17 +1168,20 @@
       <c r="G11" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H11" t="s">
-        <v>8</v>
+      <c r="H11" s="1" t="s">
+        <v>126</v>
       </c>
       <c r="I11" t="s">
         <v>8</v>
       </c>
       <c r="J11" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>21</v>
       </c>
@@ -1151,17 +1203,20 @@
       <c r="G12" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H12" t="s">
-        <v>6</v>
+      <c r="H12" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="I12" t="s">
         <v>6</v>
       </c>
       <c r="J12" t="s">
+        <v>6</v>
+      </c>
+      <c r="K12" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1183,17 +1238,20 @@
       <c r="G13" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I13" t="s">
         <v>11</v>
       </c>
-      <c r="I13" t="s">
-        <v>6</v>
-      </c>
       <c r="J13" t="s">
+        <v>6</v>
+      </c>
+      <c r="K13" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>23</v>
       </c>
@@ -1215,17 +1273,20 @@
       <c r="G14" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I14" t="s">
         <v>11</v>
       </c>
-      <c r="I14" t="s">
-        <v>6</v>
-      </c>
       <c r="J14" t="s">
+        <v>6</v>
+      </c>
+      <c r="K14" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1247,17 +1308,20 @@
       <c r="G15" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I15" t="s">
         <v>11</v>
       </c>
-      <c r="I15" t="s">
-        <v>6</v>
-      </c>
       <c r="J15" t="s">
+        <v>6</v>
+      </c>
+      <c r="K15" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -1279,17 +1343,20 @@
       <c r="G16" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I16" t="s">
         <v>11</v>
       </c>
-      <c r="I16" t="s">
-        <v>6</v>
-      </c>
       <c r="J16" t="s">
+        <v>6</v>
+      </c>
+      <c r="K16" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>26</v>
       </c>
@@ -1311,17 +1378,20 @@
       <c r="G17" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H17" t="s">
-        <v>8</v>
+      <c r="H17" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="I17" t="s">
         <v>8</v>
       </c>
       <c r="J17" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K17" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -1343,17 +1413,20 @@
       <c r="G18" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I18" t="s">
         <v>11</v>
       </c>
-      <c r="I18" t="s">
-        <v>8</v>
-      </c>
       <c r="J18" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K18" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>28</v>
       </c>
@@ -1375,17 +1448,20 @@
       <c r="G19" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H19" t="s">
-        <v>8</v>
+      <c r="H19" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="I19" t="s">
         <v>8</v>
       </c>
       <c r="J19" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K19" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -1407,17 +1483,20 @@
       <c r="G20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H20" t="s">
-        <v>8</v>
+      <c r="H20" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="I20" t="s">
         <v>8</v>
       </c>
       <c r="J20" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K20" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1439,17 +1518,20 @@
       <c r="G21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H21" t="s">
-        <v>6</v>
+      <c r="H21" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="I21" t="s">
         <v>6</v>
       </c>
       <c r="J21" t="s">
+        <v>6</v>
+      </c>
+      <c r="K21" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -1471,17 +1553,20 @@
       <c r="G22" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H22" t="s">
-        <v>8</v>
+      <c r="H22" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="I22" t="s">
         <v>8</v>
       </c>
       <c r="J22" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K22" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -1503,17 +1588,20 @@
       <c r="G23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="H23" t="s">
-        <v>6</v>
+      <c r="H23" s="1" t="s">
+        <v>126</v>
       </c>
       <c r="I23" t="s">
         <v>6</v>
       </c>
       <c r="J23" t="s">
+        <v>6</v>
+      </c>
+      <c r="K23" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>42</v>
       </c>
@@ -1535,17 +1623,20 @@
       <c r="G24" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H24" t="s">
-        <v>6</v>
-      </c>
-      <c r="I24" s="1" t="s">
+      <c r="H24" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I24" t="s">
         <v>6</v>
       </c>
       <c r="J24" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K24" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>43</v>
       </c>
@@ -1567,17 +1658,20 @@
       <c r="G25" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H25" t="s">
-        <v>6</v>
-      </c>
-      <c r="I25" s="1" t="s">
+      <c r="H25" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I25" t="s">
         <v>6</v>
       </c>
       <c r="J25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K25" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>44</v>
       </c>
@@ -1599,17 +1693,20 @@
       <c r="G26" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H26" t="s">
-        <v>6</v>
+      <c r="H26" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="I26" t="s">
         <v>6</v>
       </c>
       <c r="J26" t="s">
+        <v>6</v>
+      </c>
+      <c r="K26" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>45</v>
       </c>
@@ -1631,17 +1728,20 @@
       <c r="G27" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H27" t="s">
-        <v>8</v>
-      </c>
-      <c r="I27" s="1" t="s">
+      <c r="H27" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I27" t="s">
         <v>8</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K27" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>46</v>
       </c>
@@ -1663,17 +1763,20 @@
       <c r="G28" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H28" t="s">
-        <v>8</v>
-      </c>
-      <c r="I28" s="1" t="s">
+      <c r="H28" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I28" t="s">
         <v>8</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>47</v>
       </c>
@@ -1695,17 +1798,20 @@
       <c r="G29" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H29" t="s">
+      <c r="H29" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I29" t="s">
         <v>11</v>
       </c>
-      <c r="I29" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="J29" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K29" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>48</v>
       </c>
@@ -1727,17 +1833,20 @@
       <c r="G30" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H30" t="s">
-        <v>8</v>
-      </c>
-      <c r="I30" s="1" t="s">
+      <c r="H30" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I30" t="s">
         <v>8</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K30" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>49</v>
       </c>
@@ -1759,17 +1868,20 @@
       <c r="G31" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H31" t="s">
+      <c r="H31" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I31" t="s">
         <v>11</v>
       </c>
-      <c r="I31" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J31" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K31" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -1791,17 +1903,20 @@
       <c r="G32" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H32" t="s">
+      <c r="H32" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I32" t="s">
         <v>11</v>
       </c>
-      <c r="I32" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="J32" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K32" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>52</v>
       </c>
@@ -1823,17 +1938,20 @@
       <c r="G33" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H33" t="s">
-        <v>6</v>
-      </c>
-      <c r="I33" s="1" t="s">
+      <c r="H33" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I33" t="s">
         <v>6</v>
       </c>
       <c r="J33" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K33" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>53</v>
       </c>
@@ -1855,17 +1973,20 @@
       <c r="G34" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H34" t="s">
-        <v>8</v>
-      </c>
-      <c r="I34" s="1" t="s">
+      <c r="H34" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I34" t="s">
         <v>8</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K34" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>54</v>
       </c>
@@ -1887,17 +2008,20 @@
       <c r="G35" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H35" t="s">
+      <c r="H35" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I35" t="s">
         <v>11</v>
       </c>
-      <c r="I35" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="J35" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K35" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>55</v>
       </c>
@@ -1919,17 +2043,20 @@
       <c r="G36" t="s">
         <v>39</v>
       </c>
-      <c r="H36" t="s">
+      <c r="H36" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I36" t="s">
         <v>11</v>
       </c>
-      <c r="I36" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="J36" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K36" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>56</v>
       </c>
@@ -1951,17 +2078,20 @@
       <c r="G37" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H37" t="s">
-        <v>6</v>
-      </c>
-      <c r="I37" s="1" t="s">
+      <c r="H37" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="I37" t="s">
         <v>6</v>
       </c>
       <c r="J37" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K37" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>57</v>
       </c>
@@ -1983,17 +2113,20 @@
       <c r="G38" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H38" t="s">
-        <v>8</v>
-      </c>
-      <c r="I38" s="1" t="s">
+      <c r="H38" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I38" t="s">
         <v>8</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K38" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>58</v>
       </c>
@@ -2015,17 +2148,20 @@
       <c r="G39" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H39" t="s">
-        <v>8</v>
-      </c>
-      <c r="I39" s="1" t="s">
+      <c r="H39" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I39" t="s">
         <v>8</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K39" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>59</v>
       </c>
@@ -2047,17 +2183,20 @@
       <c r="G40" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H40" t="s">
-        <v>8</v>
-      </c>
-      <c r="I40" s="1" t="s">
+      <c r="H40" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I40" t="s">
         <v>8</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K40" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>60</v>
       </c>
@@ -2079,17 +2218,20 @@
       <c r="G41" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H41" t="s">
-        <v>8</v>
-      </c>
-      <c r="I41" s="1" t="s">
+      <c r="H41" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I41" t="s">
         <v>8</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K41" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>61</v>
       </c>
@@ -2111,17 +2253,20 @@
       <c r="G42" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H42" t="s">
-        <v>8</v>
-      </c>
-      <c r="I42" s="1" t="s">
+      <c r="H42" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I42" t="s">
         <v>8</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K42" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>62</v>
       </c>
@@ -2143,17 +2288,20 @@
       <c r="G43" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H43" t="s">
-        <v>8</v>
-      </c>
-      <c r="I43" s="1" t="s">
+      <c r="H43" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I43" t="s">
         <v>8</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K43" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>63</v>
       </c>
@@ -2175,17 +2323,20 @@
       <c r="G44" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H44" t="s">
-        <v>6</v>
-      </c>
-      <c r="I44" s="1" t="s">
+      <c r="H44" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I44" t="s">
         <v>6</v>
       </c>
       <c r="J44" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K44" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>64</v>
       </c>
@@ -2207,17 +2358,20 @@
       <c r="G45" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H45" t="s">
-        <v>8</v>
-      </c>
-      <c r="I45" s="1" t="s">
+      <c r="H45" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I45" t="s">
         <v>8</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K45" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>65</v>
       </c>
@@ -2239,17 +2393,20 @@
       <c r="G46" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H46" t="s">
-        <v>6</v>
-      </c>
-      <c r="I46" s="1" t="s">
+      <c r="H46" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I46" t="s">
         <v>6</v>
       </c>
       <c r="J46" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K46" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>66</v>
       </c>
@@ -2271,17 +2428,20 @@
       <c r="G47" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H47" t="s">
-        <v>8</v>
-      </c>
-      <c r="I47" s="1" t="s">
+      <c r="H47" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I47" t="s">
         <v>8</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K47" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>67</v>
       </c>
@@ -2303,17 +2463,20 @@
       <c r="G48" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H48" t="s">
-        <v>6</v>
-      </c>
-      <c r="I48" s="1" t="s">
+      <c r="H48" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I48" t="s">
         <v>6</v>
       </c>
       <c r="J48" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K48" s="1" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>68</v>
       </c>
@@ -2335,17 +2498,20 @@
       <c r="G49" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H49" t="s">
-        <v>6</v>
-      </c>
-      <c r="I49" s="1" t="s">
+      <c r="H49" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I49" t="s">
         <v>6</v>
       </c>
       <c r="J49" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K49" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>69</v>
       </c>
@@ -2367,17 +2533,20 @@
       <c r="G50" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H50" t="s">
+      <c r="H50" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I50" t="s">
         <v>11</v>
       </c>
-      <c r="I50" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J50" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K50" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>70</v>
       </c>
@@ -2399,17 +2568,20 @@
       <c r="G51" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H51" t="s">
+      <c r="H51" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I51" t="s">
         <v>19</v>
       </c>
-      <c r="I51" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J51" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K51" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>71</v>
       </c>
@@ -2431,17 +2603,20 @@
       <c r="G52" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H52" t="s">
-        <v>8</v>
-      </c>
-      <c r="I52" s="1" t="s">
+      <c r="H52" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I52" t="s">
         <v>8</v>
       </c>
       <c r="J52" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K52" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>72</v>
       </c>
@@ -2463,17 +2638,20 @@
       <c r="G53" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H53" t="s">
-        <v>6</v>
-      </c>
-      <c r="I53" s="1" t="s">
+      <c r="H53" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I53" t="s">
         <v>6</v>
       </c>
       <c r="J53" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K53" s="1" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>73</v>
       </c>
@@ -2495,17 +2673,20 @@
       <c r="G54" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H54" t="s">
-        <v>8</v>
-      </c>
-      <c r="I54" s="1" t="s">
+      <c r="H54" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I54" t="s">
         <v>8</v>
       </c>
       <c r="J54" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>74</v>
       </c>
@@ -2527,17 +2708,20 @@
       <c r="G55" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H55" t="s">
+      <c r="H55" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I55" t="s">
         <v>11</v>
       </c>
-      <c r="I55" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J55" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>75</v>
       </c>
@@ -2559,17 +2743,20 @@
       <c r="G56" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H56" t="s">
-        <v>8</v>
-      </c>
-      <c r="I56" s="1" t="s">
+      <c r="H56" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="I56" t="s">
         <v>8</v>
       </c>
       <c r="J56" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K56" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>76</v>
       </c>
@@ -2591,17 +2778,20 @@
       <c r="G57" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H57" t="s">
+      <c r="H57" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I57" t="s">
         <v>19</v>
       </c>
-      <c r="I57" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J57" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K57" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>77</v>
       </c>
@@ -2623,17 +2813,20 @@
       <c r="G58" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H58" t="s">
-        <v>8</v>
-      </c>
-      <c r="I58" s="1" t="s">
+      <c r="H58" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I58" t="s">
         <v>8</v>
       </c>
       <c r="J58" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K58" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>78</v>
       </c>
@@ -2655,17 +2848,20 @@
       <c r="G59" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H59" t="s">
-        <v>6</v>
-      </c>
-      <c r="I59" s="1" t="s">
+      <c r="H59" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I59" t="s">
         <v>6</v>
       </c>
       <c r="J59" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K59" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>79</v>
       </c>
@@ -2687,17 +2883,20 @@
       <c r="G60" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H60" t="s">
-        <v>8</v>
-      </c>
-      <c r="I60" s="1" t="s">
+      <c r="H60" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I60" t="s">
         <v>8</v>
       </c>
       <c r="J60" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K60" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>80</v>
       </c>
@@ -2719,17 +2918,20 @@
       <c r="G61" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H61" t="s">
+      <c r="H61" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I61" t="s">
         <v>19</v>
       </c>
-      <c r="I61" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J61" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K61" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>81</v>
       </c>
@@ -2751,17 +2953,20 @@
       <c r="G62" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H62" t="s">
-        <v>6</v>
-      </c>
-      <c r="I62" s="1" t="s">
+      <c r="H62" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I62" t="s">
         <v>6</v>
       </c>
       <c r="J62" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K62" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>82</v>
       </c>
@@ -2783,17 +2988,20 @@
       <c r="G63" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H63" t="s">
-        <v>8</v>
-      </c>
-      <c r="I63" s="1" t="s">
+      <c r="H63" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I63" t="s">
         <v>8</v>
       </c>
       <c r="J63" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K63" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>83</v>
       </c>
@@ -2815,17 +3023,20 @@
       <c r="G64" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H64" t="s">
-        <v>8</v>
-      </c>
-      <c r="I64" s="1" t="s">
+      <c r="H64" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I64" t="s">
         <v>8</v>
       </c>
       <c r="J64" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K64" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>84</v>
       </c>
@@ -2847,17 +3058,20 @@
       <c r="G65" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H65" t="s">
-        <v>6</v>
-      </c>
-      <c r="I65" s="1" t="s">
+      <c r="H65" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I65" t="s">
         <v>6</v>
       </c>
       <c r="J65" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K65" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>85</v>
       </c>
@@ -2879,17 +3093,20 @@
       <c r="G66" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H66" t="s">
-        <v>8</v>
-      </c>
-      <c r="I66" s="1" t="s">
+      <c r="H66" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I66" t="s">
         <v>8</v>
       </c>
       <c r="J66" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>86</v>
       </c>
@@ -2911,17 +3128,20 @@
       <c r="G67" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H67" t="s">
+      <c r="H67" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I67" t="s">
         <v>11</v>
       </c>
-      <c r="I67" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J67" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K67" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>87</v>
       </c>
@@ -2943,17 +3163,20 @@
       <c r="G68" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H68" t="s">
-        <v>6</v>
-      </c>
-      <c r="I68" s="1" t="s">
+      <c r="H68" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I68" t="s">
         <v>6</v>
       </c>
       <c r="J68" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K68" s="1" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>88</v>
       </c>
@@ -2975,17 +3198,20 @@
       <c r="G69" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H69" t="s">
-        <v>6</v>
-      </c>
-      <c r="I69" s="1" t="s">
+      <c r="H69" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I69" t="s">
         <v>6</v>
       </c>
       <c r="J69" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K69" s="1" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>89</v>
       </c>
@@ -3007,17 +3233,20 @@
       <c r="G70" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H70" t="s">
-        <v>8</v>
-      </c>
-      <c r="I70" s="1" t="s">
+      <c r="H70" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I70" t="s">
         <v>8</v>
       </c>
       <c r="J70" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K70" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>90</v>
       </c>
@@ -3039,17 +3268,20 @@
       <c r="G71" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H71" t="s">
-        <v>8</v>
-      </c>
-      <c r="I71" s="1" t="s">
+      <c r="H71" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I71" t="s">
         <v>8</v>
       </c>
       <c r="J71" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K71" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>91</v>
       </c>
@@ -3071,17 +3303,20 @@
       <c r="G72" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H72" t="s">
-        <v>8</v>
-      </c>
-      <c r="I72" s="1" t="s">
+      <c r="H72" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I72" t="s">
         <v>8</v>
       </c>
       <c r="J72" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>92</v>
       </c>
@@ -3103,17 +3338,20 @@
       <c r="G73" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H73" t="s">
-        <v>8</v>
-      </c>
-      <c r="I73" s="1" t="s">
+      <c r="H73" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I73" t="s">
         <v>8</v>
       </c>
       <c r="J73" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>93</v>
       </c>
@@ -3135,17 +3373,20 @@
       <c r="G74" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H74" t="s">
+      <c r="H74" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="I74" t="s">
         <v>19</v>
       </c>
-      <c r="I74" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J74" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K74" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>94</v>
       </c>
@@ -3167,17 +3408,20 @@
       <c r="G75" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H75" t="s">
+      <c r="H75" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I75" t="s">
         <v>11</v>
       </c>
-      <c r="I75" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J75" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K75" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>95</v>
       </c>
@@ -3199,17 +3443,20 @@
       <c r="G76" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H76" t="s">
+      <c r="H76" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I76" t="s">
         <v>19</v>
       </c>
-      <c r="I76" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J76" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>96</v>
       </c>
@@ -3231,17 +3478,20 @@
       <c r="G77" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H77" t="s">
-        <v>8</v>
-      </c>
-      <c r="I77" s="1" t="s">
+      <c r="H77" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I77" t="s">
         <v>8</v>
       </c>
       <c r="J77" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K77" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>97</v>
       </c>
@@ -3263,17 +3513,20 @@
       <c r="G78" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H78" t="s">
-        <v>8</v>
-      </c>
-      <c r="I78" s="1" t="s">
+      <c r="H78" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I78" t="s">
         <v>8</v>
       </c>
       <c r="J78" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K78" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>98</v>
       </c>
@@ -3295,17 +3548,20 @@
       <c r="G79" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H79" t="s">
-        <v>8</v>
-      </c>
-      <c r="I79" s="1" t="s">
+      <c r="H79" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I79" t="s">
         <v>8</v>
       </c>
       <c r="J79" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K79" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>99</v>
       </c>
@@ -3327,17 +3583,20 @@
       <c r="G80" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H80" t="s">
-        <v>8</v>
-      </c>
-      <c r="I80" s="1" t="s">
+      <c r="H80" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I80" t="s">
         <v>8</v>
       </c>
       <c r="J80" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K80" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>100</v>
       </c>
@@ -3359,17 +3618,20 @@
       <c r="G81" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H81" t="s">
-        <v>8</v>
-      </c>
-      <c r="I81" s="1" t="s">
+      <c r="H81" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I81" t="s">
         <v>8</v>
       </c>
       <c r="J81" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>102</v>
       </c>
@@ -3391,17 +3653,20 @@
       <c r="G82" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H82" t="s">
-        <v>8</v>
-      </c>
-      <c r="I82" s="1" t="s">
+      <c r="H82" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I82" t="s">
         <v>8</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K82" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>101</v>
       </c>
@@ -3423,17 +3688,20 @@
       <c r="G83" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H83" t="s">
+      <c r="H83" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I83" t="s">
         <v>19</v>
       </c>
-      <c r="I83" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J83" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K83" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>103</v>
       </c>
@@ -3455,17 +3723,20 @@
       <c r="G84" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H84" t="s">
-        <v>6</v>
-      </c>
-      <c r="I84" s="1" t="s">
+      <c r="H84" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I84" t="s">
         <v>6</v>
       </c>
       <c r="J84" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K84" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>104</v>
       </c>
@@ -3487,17 +3758,20 @@
       <c r="G85" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H85" t="s">
-        <v>8</v>
-      </c>
-      <c r="I85" s="1" t="s">
+      <c r="H85" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I85" t="s">
         <v>8</v>
       </c>
       <c r="J85" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K85" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>105</v>
       </c>
@@ -3519,17 +3793,20 @@
       <c r="G86" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H86" t="s">
-        <v>8</v>
-      </c>
-      <c r="I86" s="1" t="s">
+      <c r="H86" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I86" t="s">
         <v>8</v>
       </c>
       <c r="J86" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K86" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>106</v>
       </c>
@@ -3551,17 +3828,20 @@
       <c r="G87" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H87" t="s">
-        <v>6</v>
-      </c>
-      <c r="I87" s="1" t="s">
+      <c r="H87" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="I87" t="s">
         <v>6</v>
       </c>
       <c r="J87" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K87" s="1" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>107</v>
       </c>
@@ -3583,17 +3863,20 @@
       <c r="G88" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H88" t="s">
-        <v>6</v>
-      </c>
-      <c r="I88" s="1" t="s">
+      <c r="H88" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I88" t="s">
         <v>6</v>
       </c>
       <c r="J88" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="K88" s="1" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>110</v>
       </c>
@@ -3615,17 +3898,20 @@
       <c r="G89" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="H89" t="s">
+      <c r="H89" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I89" t="s">
         <v>11</v>
       </c>
-      <c r="I89" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J89" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K89" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>108</v>
       </c>
@@ -3647,17 +3933,20 @@
       <c r="G90" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H90" t="s">
+      <c r="H90" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I90" t="s">
         <v>19</v>
       </c>
-      <c r="I90" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J90" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K90" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>109</v>
       </c>
@@ -3679,17 +3968,20 @@
       <c r="G91" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="H91" t="s">
-        <v>8</v>
-      </c>
-      <c r="I91" s="1" t="s">
+      <c r="H91" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I91" t="s">
         <v>8</v>
       </c>
       <c r="J91" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
+        <v>8</v>
+      </c>
+      <c r="K91" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>111</v>
       </c>
@@ -3711,13 +4003,16 @@
       <c r="G92" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H92" t="s">
+      <c r="H92" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I92" t="s">
         <v>19</v>
       </c>
-      <c r="I92" s="1" t="s">
-        <v>8</v>
-      </c>
       <c r="J92" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K92" s="1" t="s">
         <v>117</v>
       </c>
     </row>

</xml_diff>